<commit_message>
feat: add match session lifecycle
- Add match container, Lua builtins, and per-type scripts
- Carry match id/type on transfer login flags
- Instance maps by match slot and hook death/disconnect
- Add matchmaking map DSL and match maps
</commit_message>
<xml_diff>
--- a/resources/table/matchmaking.xlsx
+++ b/resources/table/matchmaking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91BC895A-B103-4F7D-9377-B7E1B2611D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3945BDA6-477B-41A7-8A1A-A8BA263F7636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
   </bookViews>
   <sheets>
     <sheet name="matchmaking" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -57,6 +57,21 @@
   <si>
     <t>team_count</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>map</t>
+  </si>
+  <si>
+    <t>dsl</t>
+  </si>
+  <si>
+    <t>server</t>
+  </si>
+  <si>
+    <t>map(616, 10, 10, 20, 20)</t>
+  </si>
+  <si>
+    <t>map(616, 15, 3)</t>
   </si>
 </sst>
 </file>
@@ -434,16 +449,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE8D9647-70DB-4352-ABD3-4D2F60838B15}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9" style="1"/>
+    <col min="4" max="4" width="20.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -453,8 +469,11 @@
       <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -464,8 +483,11 @@
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -475,8 +497,11 @@
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -486,8 +511,11 @@
       <c r="C4" s="1">
         <v>2</v>
       </c>
+      <c r="D4" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -497,8 +525,11 @@
       <c r="C5" s="1">
         <v>2</v>
       </c>
+      <c r="D5" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
     </row>
   </sheetData>

</xml_diff>